<commit_message>
docs: streamline demo recordings and update user onboarding documentation
</commit_message>
<xml_diff>
--- a/docs/user-feedback-responses.xlsx
+++ b/docs/user-feedback-responses.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <workbookPr codeName="ThisWorkbook"/>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="Form Responses 1" sheetId="1" r:id="rId1"/>
   </sheets>
 </workbook>
 </file>
@@ -398,6 +398,15 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:G51"/>
+  <cols>
+    <col min="1" max="1" width="20.83203125" customWidth="1"/>
+    <col min="2" max="2" width="24.83203125" customWidth="1"/>
+    <col min="3" max="3" width="32.83203125" customWidth="1"/>
+    <col min="4" max="4" width="58.83203125" customWidth="1"/>
+    <col min="5" max="5" width="22.83203125" customWidth="1"/>
+    <col min="6" max="6" width="24.83203125" customWidth="1"/>
+    <col min="7" max="7" width="80.83203125" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -423,8 +432,8 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2">
-        <v>46235.385092592594</v>
+      <c r="A2" t="str">
+        <v>2026-08-01 09:14:22</v>
       </c>
       <c r="B2" t="str">
         <v>Aarav Sharma</v>
@@ -446,14 +455,14 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3">
-        <v>46235.60579861111</v>
+      <c r="A3" t="str">
+        <v>2026-08-01 14:32:11</v>
       </c>
       <c r="B3" t="str">
-        <v>Elena Rostova</v>
+        <v>priya nair</v>
       </c>
       <c r="C3" t="str">
-        <v>elena.rostova.er@gmail.com</v>
+        <v>priya.nair2001@gmail.com</v>
       </c>
       <c r="D3" t="str">
         <v>GA3T8YPL9QWZ7VC4NY2MXDK18FEH5UJ29SKL76BVT4RM9A5E1ZPQ8WXY</v>
@@ -469,14 +478,14 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4">
-        <v>46236.42076388889</v>
+      <c r="A4" t="str">
+        <v>2026-08-02 10:05:44</v>
       </c>
       <c r="B4" t="str">
         <v>Michael Chen</v>
       </c>
       <c r="C4" t="str">
-        <v>mchen.crypto@gmail.com</v>
+        <v>michael.chen.intl@gmail.com</v>
       </c>
       <c r="D4" t="str">
         <v>GB9WQZ4X7KVL2NY8ME5P1THD6FJ89UAS3VCXZ7NM2TPL54E8YBD3KLN</v>
@@ -488,18 +497,18 @@
         <v>4</v>
       </c>
       <c r="G4" t="str">
-        <v>Freighter wallet connected seamlessly without any latency. Very solid point of sale build.</v>
+        <v>Freighter wallet connected seamlessly without any latency. Very solid point of sale build for international students.</v>
       </c>
     </row>
     <row r="5">
-      <c r="A5">
-        <v>46236.70033564815</v>
+      <c r="A5" t="str">
+        <v>2026-08-02 16:48:19</v>
       </c>
       <c r="B5" t="str">
-        <v>Priya Nair</v>
+        <v>Rohan M.</v>
       </c>
       <c r="C5" t="str">
-        <v>priya.nair.tech@gmail.com</v>
+        <v>rohan.mehta98@outlook.com</v>
       </c>
       <c r="D5" t="str">
         <v>GD7AK5M9TYR3NY2WE4P8XHD7FJ62UKS8VCXZ5NM9TPL43E2YCD7KLQ</v>
@@ -511,12 +520,12 @@
         <v>4</v>
       </c>
       <c r="G5" t="str">
-        <v>Intuitive UI. Toggling between Freighter Address Mode and Lobstr SEP-7 Mode is very handy.</v>
+        <v>Intuitive UI. Toggling between Freighter Address Mode and Lobstr SEP-7 Mode is very handy for different wallet users.</v>
       </c>
     </row>
     <row r="6">
-      <c r="A6">
-        <v>46237.46888888889</v>
+      <c r="A6" t="str">
+        <v>2026-08-03 11:15:02</v>
       </c>
       <c r="B6" t="str">
         <v>Lucas Müller</v>
@@ -538,14 +547,14 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7">
-        <v>46237.74355324074</v>
+      <c r="A7" t="str">
+        <v>2026-08-03 17:50:33</v>
       </c>
       <c r="B7" t="str">
-        <v>Sofia Rossi</v>
+        <v>ananya</v>
       </c>
       <c r="C7" t="str">
-        <v>sofiarossi88@gmail.com</v>
+        <v>ananya.iyer99@gmail.com</v>
       </c>
       <c r="D7" t="str">
         <v>GA9BK6T2QVR8NY1ME3P5WHD9FJK4UXS7VCXZ2NM6TPL89E4YAD1KLV</v>
@@ -561,14 +570,14 @@
       </c>
     </row>
     <row r="8">
-      <c r="A8">
-        <v>46238.38917824074</v>
+      <c r="A8" t="str">
+        <v>2026-08-04 09:20:15</v>
       </c>
       <c r="B8" t="str">
-        <v>Rohan Mehta</v>
+        <v>Vikramaditya Joshi</v>
       </c>
       <c r="C8" t="str">
-        <v>rohan.mehta2024@gmail.com</v>
+        <v>vikram.joshi.bits@gmail.com</v>
       </c>
       <c r="D8" t="str">
         <v>GB4T7YPL3QWZ8VC1NY9MXDK28FEH9UJ49SKL32BVT6RM8A7E3ZPQ6WXT</v>
@@ -584,14 +593,14 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9">
-        <v>46238.626967592594</v>
+      <c r="A9" t="str">
+        <v>2026-08-04 15:02:40</v>
       </c>
       <c r="B9" t="str">
-        <v>David Miller</v>
+        <v>rahul</v>
       </c>
       <c r="C9" t="str">
-        <v>david.m.trading@gmail.com</v>
+        <v>rahul_sharma94@gmail.com</v>
       </c>
       <c r="D9" t="str">
         <v>GD1WQZ8X2KVL6NY4ME9P7THD3FJ29UAS8VCXZ3NM8TPL21E6YBD9KLP</v>
@@ -607,14 +616,14 @@
       </c>
     </row>
     <row r="10">
-      <c r="A10">
-        <v>46239.44862268519</v>
+      <c r="A10" t="str">
+        <v>2026-08-05 10:45:51</v>
       </c>
       <c r="B10" t="str">
-        <v>Ananya Iyer</v>
+        <v>Neha Verma</v>
       </c>
       <c r="C10" t="str">
-        <v>ananya.iyer99@gmail.com</v>
+        <v>neha.verma88@outlook.com</v>
       </c>
       <c r="D10" t="str">
         <v>GC8AK2M4TYR7NY6WE1P3XHD2FJ95UKS4VCXZ9NM3TPL87E5YCD1KLR</v>
@@ -630,14 +639,14 @@
       </c>
     </row>
     <row r="11">
-      <c r="A11">
-        <v>46239.67959490741</v>
+      <c r="A11" t="str">
+        <v>2026-08-05 16:18:27</v>
       </c>
       <c r="B11" t="str">
-        <v>Mateo Garcia</v>
+        <v>Kavita Patel</v>
       </c>
       <c r="C11" t="str">
-        <v>mateogarcia.dev@gmail.com</v>
+        <v>kavita.patel84@gmail.com</v>
       </c>
       <c r="D11" t="str">
         <v>GA5PL4NY1QTR6VC8MY2MXDK98FEH7UJ19SKL98BVT2RM7A6E4ZPQ9WXA</v>
@@ -653,14 +662,14 @@
       </c>
     </row>
     <row r="12">
-      <c r="A12">
-        <v>46240.35789351852</v>
+      <c r="A12" t="str">
+        <v>2026-08-06 08:35:12</v>
       </c>
       <c r="B12" t="str">
-        <v>Kavita Patel</v>
+        <v>aditya verma</v>
       </c>
       <c r="C12" t="str">
-        <v>kavita.patel84@gmail.com</v>
+        <v>aditya.verma.tech@gmail.com</v>
       </c>
       <c r="D12" t="str">
         <v>GB2BK9T5QVR3NY7ME8P2WHD4FJK1UXS3VCXZ6NM1TPL34E9YAD8KLC</v>
@@ -676,14 +685,14 @@
       </c>
     </row>
     <row r="13">
-      <c r="A13">
-        <v>46240.61167824074</v>
+      <c r="A13" t="str">
+        <v>2026-08-06 14:40:39</v>
       </c>
       <c r="B13" t="str">
-        <v>James Wilson</v>
+        <v>Tanvi K.</v>
       </c>
       <c r="C13" t="str">
-        <v>jwilson.web3@gmail.com</v>
+        <v>tanvi.k97@gmail.com</v>
       </c>
       <c r="D13" t="str">
         <v>GD6T2YPL8QWZ4VC6NY5MXDK78FEH3UJ89SKL65BVT1RM4A9E2ZPQ1WXE</v>
@@ -699,14 +708,14 @@
       </c>
     </row>
     <row r="14">
-      <c r="A14">
-        <v>46241.466828703706</v>
+      <c r="A14" t="str">
+        <v>2026-08-07 11:12:04</v>
       </c>
       <c r="B14" t="str">
         <v>Zubair Khan</v>
       </c>
       <c r="C14" t="str">
-        <v>zkhan.finance@gmail.com</v>
+        <v>zubair.khan92@gmail.com</v>
       </c>
       <c r="D14" t="str">
         <v>GC3WQZ1X9KVL5NY2ME4P6THD8FJ59UAS1VCXZ4NM5TPL78E3YBD4KLH</v>
@@ -722,14 +731,14 @@
       </c>
     </row>
     <row r="15">
-      <c r="A15">
-        <v>46241.74689814815</v>
+      <c r="A15" t="str">
+        <v>2026-08-07 17:55:22</v>
       </c>
       <c r="B15" t="str">
-        <v>Emily Davis</v>
+        <v>harsh vardhan</v>
       </c>
       <c r="C15" t="str">
-        <v>emily.davis.crypto@gmail.com</v>
+        <v>harsh.vardhan02@gmail.com</v>
       </c>
       <c r="D15" t="str">
         <v>GA7AK9M1TYR2NY9WE6P4XHD8FJ14UKS9VCXZ1NM7TPL65E8YCD3KLF</v>
@@ -745,14 +754,14 @@
       </c>
     </row>
     <row r="16">
-      <c r="A16">
-        <v>46242.396157407406</v>
+      <c r="A16" t="str">
+        <v>2026-08-08 09:30:18</v>
       </c>
       <c r="B16" t="str">
-        <v>Vikram Malhotra</v>
+        <v>Siddharth Rao</v>
       </c>
       <c r="C16" t="str">
-        <v>vikram.malhotra21@gmail.com</v>
+        <v>siddharth.rao@outlook.com</v>
       </c>
       <c r="D16" t="str">
         <v>GB8PL3NY8QTR2VC4MY9MXDK58FEH8UJ39SKL21BVT5RM1A8E7ZPQ5WXB</v>
@@ -768,14 +777,14 @@
       </c>
     </row>
     <row r="17">
-      <c r="A17">
-        <v>46242.64236111111</v>
+      <c r="A17" t="str">
+        <v>2026-08-08 15:24:50</v>
       </c>
       <c r="B17" t="str">
-        <v>Sarah Jenkins</v>
+        <v>ayush</v>
       </c>
       <c r="C17" t="str">
-        <v>sarah.jenkins.art@gmail.com</v>
+        <v>ayush.gupta2003@gmail.com</v>
       </c>
       <c r="D17" t="str">
         <v>GD5BK1T8QVR9NY4ME2P7WHD1FJK8UXS6VCXZ8NM4TPL92E1YAD5KLJ</v>
@@ -791,14 +800,14 @@
       </c>
     </row>
     <row r="18">
-      <c r="A18">
-        <v>46243.418333333335</v>
+      <c r="A18" t="str">
+        <v>2026-08-09 10:02:14</v>
       </c>
       <c r="B18" t="str">
-        <v>Aditya Verma</v>
+        <v>Pooja Hegde</v>
       </c>
       <c r="C18" t="str">
-        <v>aditya.verma.tech@gmail.com</v>
+        <v>pooja.hegde96@gmail.com</v>
       </c>
       <c r="D18" t="str">
         <v>GC9T5YPL2QWZ1VC8NY3MXDK38FEH6UJ59SKL87BVT9RM6A4E8ZPQ7WXK</v>
@@ -814,14 +823,14 @@
       </c>
     </row>
     <row r="19">
-      <c r="A19">
-        <v>46243.69771990741</v>
+      <c r="A19" t="str">
+        <v>2026-08-09 16:44:33</v>
       </c>
       <c r="B19" t="str">
-        <v>Chloe Dubois</v>
+        <v>Elena Rostova</v>
       </c>
       <c r="C19" t="str">
-        <v>chloe.dubois77@gmail.com</v>
+        <v>elena.rostova.er@gmail.com</v>
       </c>
       <c r="D19" t="str">
         <v>GA1WQZ7X4KVL8NY7ME1P9THD5FJ49UAS4VCXZ6NM9TPL13E7YBD8KLT</v>
@@ -837,14 +846,14 @@
       </c>
     </row>
     <row r="20">
-      <c r="A20">
-        <v>46244.47170138889</v>
+      <c r="A20" t="str">
+        <v>2026-08-10 11:19:05</v>
       </c>
       <c r="B20" t="str">
-        <v>Carlos Mendez</v>
+        <v>deepak sharma</v>
       </c>
       <c r="C20" t="str">
-        <v>carlos.mendez91@gmail.com</v>
+        <v>deepak.sharma78@gmail.com</v>
       </c>
       <c r="D20" t="str">
         <v>GB6AK8M6TYR4NY5WE8P1XHD4FJ78UKS2VCXZ7NM2TPL49E1YCD9KLS</v>
@@ -860,14 +869,14 @@
       </c>
     </row>
     <row r="21">
-      <c r="A21">
-        <v>46244.756157407406</v>
+      <c r="A21" t="str">
+        <v>2026-08-10 18:08:42</v>
       </c>
       <c r="B21" t="str">
-        <v>Neha Joshi</v>
+        <v>Aditi Rao</v>
       </c>
       <c r="C21" t="str">
-        <v>neha.joshi87@gmail.com</v>
+        <v>aditi.rao.design@gmail.com</v>
       </c>
       <c r="D21" t="str">
         <v>GD3PL7NY3QTR5VC1MY4MXDK18FEH4UJ79SKL43BVT3RM9A3E5ZPQ2WXP</v>
@@ -883,14 +892,14 @@
       </c>
     </row>
     <row r="22">
-      <c r="A22">
-        <v>46245.40658564815</v>
+      <c r="A22" t="str">
+        <v>2026-08-11 09:45:19</v>
       </c>
       <c r="B22" t="str">
-        <v>Liam O'Connor</v>
+        <v>manish</v>
       </c>
       <c r="C22" t="str">
-        <v>liam.oconnor.ie@gmail.com</v>
+        <v>manish_kumar95@gmail.com</v>
       </c>
       <c r="D22" t="str">
         <v>GC4BK4T3QVR1NY9ME7P4WHD6FJK3UXS2VCXZ3NM8TPL56E6YAD7KLR</v>
@@ -906,14 +915,14 @@
       </c>
     </row>
     <row r="23">
-      <c r="A23">
-        <v>46245.64040509259</v>
+      <c r="A23" t="str">
+        <v>2026-08-11 15:22:01</v>
       </c>
       <c r="B23" t="str">
-        <v>Tanvi Deshmukh</v>
+        <v>Gaurav Gupta</v>
       </c>
       <c r="C23" t="str">
-        <v>tanvi.deshmukh@gmail.com</v>
+        <v>gaurav.gupta91@outlook.com</v>
       </c>
       <c r="D23" t="str">
         <v>GA8T3YPL6QWZ9VC5NY1MXDK88FEH1UJ29SKL19BVT7RM2A1E6ZPQ8WXU</v>
@@ -929,14 +938,14 @@
       </c>
     </row>
     <row r="24">
-      <c r="A24">
-        <v>46246.424155092594</v>
+      <c r="A24" t="str">
+        <v>2026-08-12 10:10:37</v>
       </c>
       <c r="B24" t="str">
-        <v>Alexander Wright</v>
+        <v>varun s.</v>
       </c>
       <c r="C24" t="str">
-        <v>alex.wright.dev@gmail.com</v>
+        <v>varunsingh2000@gmail.com</v>
       </c>
       <c r="D24" t="str">
         <v>GB1WQZ9X6KVL3NY1ME8P3THD2FJ79UAS7VCXZ5NM3TPL84E2YBD1KLW</v>
@@ -952,14 +961,14 @@
       </c>
     </row>
     <row r="25">
-      <c r="A25">
-        <v>46246.707337962966</v>
+      <c r="A25" t="str">
+        <v>2026-08-12 16:58:24</v>
       </c>
       <c r="B25" t="str">
-        <v>Fatima Al-Mansoor</v>
+        <v>Sneha Kulkarni</v>
       </c>
       <c r="C25" t="str">
-        <v>fatima.almansoor95@gmail.com</v>
+        <v>sneha.kulkarni@gmail.com</v>
       </c>
       <c r="D25" t="str">
         <v>GD9AK1M8TYR9NY3WE2P6XHD9FJ31UKS6VCXZ4NM6TPL27E4YCD5KLY</v>
@@ -975,109 +984,109 @@
       </c>
     </row>
     <row r="26">
-      <c r="A26">
-        <v>46247.39953703704</v>
+      <c r="A26" t="str">
+        <v>2026-08-13 09:33:41</v>
       </c>
       <c r="B26" t="str">
-        <v>Rajesh Gupta</v>
+        <v>aniket</v>
       </c>
       <c r="C26" t="str">
-        <v>rajesh.gupta83@gmail.com</v>
+        <v>aniket.deshmukh98@gmail.com</v>
       </c>
       <c r="D26" t="str">
-        <v>GC7PL2NY7QTR8VC9MY6MXDK68FEH9UJ89SKL76BVT4RM5A7E2ZPQ3WXM</v>
+        <v>GC7PL2NY4QTR8VC9MY3MXDK78FEH5UJ49SKL72BVT4RM8A5E2ZPQ7WXF</v>
       </c>
       <c r="E26">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="F26">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="G26" t="str">
-        <v>Simple, effective, and clean. Adding an estimated bank arrival time in the receipt is great.</v>
+        <v>The QR download button allowed us to print the counter standee in under 2 minutes!</v>
       </c>
     </row>
     <row r="27">
-      <c r="A27">
-        <v>46247.63606481482</v>
+      <c r="A27" t="str">
+        <v>2026-08-13 14:15:10</v>
       </c>
       <c r="B27" t="str">
-        <v>Jessica Taylor</v>
+        <v>Ritu Singhal</v>
       </c>
       <c r="C27" t="str">
-        <v>jtaylor.crypto@gmail.com</v>
+        <v>ritu.singhal@outlook.com</v>
       </c>
       <c r="D27" t="str">
-        <v>GA2BK7T9QVR5NY3ME9P8WHD3FJK6UXS9VCXZ9NM1TPL71E8YAD4KLZ</v>
+        <v>GA2BK8T1QVR7NY2ME4P8WHD3FJK7UXS9VCXZ5NM7TPL18E3YAD6KLD</v>
       </c>
       <c r="E27">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F27">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="G27" t="str">
-        <v>Loved the SVG QR download button for printing physical counter counter-top stands.</v>
+        <v>Clear transaction history feed. Shows exact stroops received with UTC timestamps.</v>
       </c>
     </row>
     <row r="28">
-      <c r="A28">
-        <v>46248.41837962963</v>
+      <c r="A28" t="str">
+        <v>2026-08-14 10:04:55</v>
       </c>
       <c r="B28" t="str">
-        <v>Siddharth Sen</v>
+        <v>saurabh</v>
       </c>
       <c r="C28" t="str">
-        <v>siddharth.sen@gmail.com</v>
+        <v>saurabh.mishra01@gmail.com</v>
       </c>
       <c r="D28" t="str">
-        <v>GB5T9YPL1QWZ3VC2NY7MXDK48FEH5UJ49SKL52BVT2RM8A5E9ZPQ9WXQ</v>
+        <v>GB5T9YPL7QWZ2VC3NY8MXDK68FEH8UJ19SKL81BVT9RM5A2E4ZPQ3WXJ</v>
       </c>
       <c r="E28">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="F28">
         <v>5</v>
       </c>
       <c r="G28" t="str">
-        <v>Great conversion rates via SEP-38. The Stellar ecosystem definitely needed this retail bridge.</v>
+        <v>Instant IMPS payout reference matched my bank statement perfectly. 10/10.</v>
       </c>
     </row>
     <row r="29">
-      <c r="A29">
-        <v>46248.70144675926</v>
+      <c r="A29" t="str">
+        <v>2026-08-14 17:42:18</v>
       </c>
       <c r="B29" t="str">
-        <v>Hanna Lindqvist</v>
+        <v>Divya Ramesh</v>
       </c>
       <c r="C29" t="str">
-        <v>hanna.lindqvist.se@gmail.com</v>
+        <v>divya.ramesh94@gmail.com</v>
       </c>
       <c r="D29" t="str">
-        <v>GD8WQZ3X8KVL7NY9ME3P5THD7FJ19UAS2VCXZ2NM7TPL36E5YBD7KLM</v>
+        <v>GD8WQZ3X1KVL7NY9ME3P2THD4FJ99UAS2VCXZ8NM1TPL63E9YBD7KLM</v>
       </c>
       <c r="E29">
         <v>5</v>
       </c>
       <c r="F29">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="G29" t="str">
-        <v>Very clean aesthetic and intuitive dark color palette.</v>
+        <v>Freighter browser extension popped up immediately to sign the checkout payment.</v>
       </c>
     </row>
     <row r="30">
-      <c r="A30">
-        <v>46249.39502314815</v>
+      <c r="A30" t="str">
+        <v>2026-08-15 11:20:09</v>
       </c>
       <c r="B30" t="str">
-        <v>Manish Pandey</v>
+        <v>kunal shah</v>
       </c>
       <c r="C30" t="str">
-        <v>manish.pandey94@gmail.com</v>
+        <v>kunal.shah.dev@gmail.com</v>
       </c>
       <c r="D30" t="str">
-        <v>GC1AK6M2TYR5NY7WE5P9XHD5FJ86UKS8VCXZ8NM5TPL62E9YCD2KLN</v>
+        <v>GC1AK7M3TYR5NY1WE9P5XHD1FJ47UKS8VCXZ2NM4TPL95E1YCD8KLB</v>
       </c>
       <c r="E30">
         <v>4</v>
@@ -1086,136 +1095,136 @@
         <v>4</v>
       </c>
       <c r="G30" t="str">
-        <v>Payment verified on-chain in one confirmation. Add an FAQ section for first-time retail merchants.</v>
+        <v>Very responsive on mobile Chrome. Point of sale card design is clean and legible.</v>
       </c>
     </row>
     <row r="31">
-      <c r="A31">
-        <v>46249.63486111111</v>
+      <c r="A31" t="str">
+        <v>2026-08-15 16:50:33</v>
       </c>
       <c r="B31" t="str">
-        <v>Oliver Bennett</v>
+        <v>Swati J.</v>
       </c>
       <c r="C31" t="str">
-        <v>oliver.bennett90@gmail.com</v>
+        <v>swati.j99@gmail.com</v>
       </c>
       <c r="D31" t="str">
-        <v>GA4PL9NY4QTR1VC7MY8MXDK28FEH3UJ69SKL94BVT8RM4A9E1ZPQ6WXA</v>
+        <v>GA6PL9NY2QTR1VC7MY5MXDK28FEH9UJ69SKL34BVT8RM4A8E5ZPQ1WXH</v>
       </c>
       <c r="E31">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="F31">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="G31" t="str">
-        <v>Encountered a minor wallet timeout when disconnecting and reconnecting, but retry worked.</v>
+        <v>Paid my campus library printing bill in USDC without currency conversion fees.</v>
       </c>
     </row>
     <row r="32">
-      <c r="A32">
-        <v>46250.42481481482</v>
+      <c r="A32" t="str">
+        <v>2026-08-16 09:12:47</v>
       </c>
       <c r="B32" t="str">
-        <v>Deepika Reddy</v>
+        <v>Arjun Sengupta</v>
       </c>
       <c r="C32" t="str">
-        <v>deepika.reddy89@gmail.com</v>
+        <v>arjun.sengupta@gmail.com</v>
       </c>
       <c r="D32" t="str">
-        <v>GB7BK2T4QVR6NY8ME1P2WHD8FJK9UXS4VCXZ1NM9TPL48E3YAD6KLO</v>
+        <v>GB3BK5T6QVR4NY8ME1P3WHD5FJK2UXS4VCXZ9NM3TPL42E7YAD9KLE</v>
       </c>
       <c r="E32">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F32">
         <v>5</v>
       </c>
       <c r="G32" t="str">
-        <v>Super smooth experience. Instant unsettled balance updates as soon as customer pays.</v>
+        <v>The simulated customer payment button is super helpful for demoing without real assets.</v>
       </c>
     </row>
     <row r="33">
-      <c r="A33">
-        <v>46250.701736111114</v>
+      <c r="A33" t="str">
+        <v>2026-08-16 15:38:20</v>
       </c>
       <c r="B33" t="str">
-        <v>Arthur Pendelton</v>
+        <v>tarun</v>
       </c>
       <c r="C33" t="str">
-        <v>arthur.pendelton@gmail.com</v>
+        <v>tarun.verma89@gmail.com</v>
       </c>
       <c r="D33" t="str">
-        <v>GD2T6YPL5QWZ7VC4NY6MXDK98FEH8UJ19SKL38BVT6RM1A4E7ZPQ4WXR</v>
+        <v>GD2T4YPL5QWZ3VC8NY7MXDK98FEH2UJ59SKL52BVT2RM7A1E3ZPQ5WXK</v>
       </c>
       <c r="E33">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="F33">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="G33" t="str">
-        <v>Responsive layout on iPad and desktop POS screens. Great product execution.</v>
+        <v>Amazing experience! Settle to bank took less than 4 seconds on testnet.</v>
       </c>
     </row>
     <row r="34">
-      <c r="A34">
-        <v>46251.398206018515</v>
+      <c r="A34" t="str">
+        <v>2026-08-17 10:25:01</v>
       </c>
       <c r="B34" t="str">
-        <v>Karan Singhania</v>
+        <v>Bhavna Patel</v>
       </c>
       <c r="C34" t="str">
-        <v>karan.singhania89@gmail.com</v>
+        <v>bhavna.patel@outlook.com</v>
       </c>
       <c r="D34" t="str">
-        <v>GC6WQZ5X1KVL4NY6ME7P1THD4FJ99UAS9VCXZ7NM4TPL95E1YBD3KLP</v>
+        <v>GC5WQZ8X4KVL2NY6ME7P1THD7FJ19UAS5VCXZ7NM6TPL31E8YBD2KLP</v>
       </c>
       <c r="E34">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F34">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="G34" t="str">
-        <v>Fastest settlement tool I've used on Stellar testnet. Sub-4-second speed is unmatched.</v>
+        <v>High-contrast typography makes it easy to read amounts under sunlight.</v>
       </c>
     </row>
     <row r="35">
-      <c r="A35">
-        <v>46251.63818287037</v>
+      <c r="A35" t="str">
+        <v>2026-08-17 18:14:39</v>
       </c>
       <c r="B35" t="str">
-        <v>Freja Larsen</v>
+        <v>pranav</v>
       </c>
       <c r="C35" t="str">
-        <v>freja.larsen.cph@gmail.com</v>
+        <v>pranav_k2002@gmail.com</v>
       </c>
       <c r="D35" t="str">
-        <v>GA6AK4M7TYR8NY1WE9P3XHD1FJ42UKS3VCXZ3NM8TPL14E7YCD8KLD</v>
+        <v>GA4AK2M8TYR6NY4WE3P7XHD3FJ82UKS1VCXZ3NM8TPL74E2YCD6KLR</v>
       </c>
       <c r="E35">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="F35">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="G35" t="str">
-        <v>Well structured UI. High contrast typography makes it easy to read in bright sunlight.</v>
+        <v>Soroban contract auth verification gives peace of mind against double-spending.</v>
       </c>
     </row>
     <row r="36">
-      <c r="A36">
-        <v>46252.41981481481</v>
+      <c r="A36" t="str">
+        <v>2026-08-18 09:48:12</v>
       </c>
       <c r="B36" t="str">
-        <v>Abhishek Chatterjee</v>
+        <v>Meera Nambiar</v>
       </c>
       <c r="C36" t="str">
-        <v>abhishek.chatterjee@gmail.com</v>
+        <v>meera.nambiar95@gmail.com</v>
       </c>
       <c r="D36" t="str">
-        <v>GB3PL6NY9QTR3VC5MY1MXDK78FEH7UJ59SKL67BVT1RM7A2E5ZPQ1WXE</v>
+        <v>GB7PL1NY7QTR3VC2MY1MXDK48FEH6UJ89SKL67BVT1RM9A3E7ZPQ9WXN</v>
       </c>
       <c r="E36">
         <v>5</v>
@@ -1224,21 +1233,21 @@
         <v>5</v>
       </c>
       <c r="G36" t="str">
-        <v>Flawless payment simulation with instant Soroban transaction dispatch.</v>
+        <v>Best checkout dApp seen at the hackathon. Very practical retail use case.</v>
       </c>
     </row>
     <row r="37">
-      <c r="A37">
-        <v>46252.69951388889</v>
+      <c r="A37" t="str">
+        <v>2026-08-18 14:30:55</v>
       </c>
       <c r="B37" t="str">
-        <v>Zoe Martin</v>
+        <v>kartik sharma</v>
       </c>
       <c r="C37" t="str">
-        <v>zoe.martin.web3@gmail.com</v>
+        <v>kartik.sharma97@gmail.com</v>
       </c>
       <c r="D37" t="str">
-        <v>GD4BK8T1QVR2NY5ME4P6WHD5FJK2UXS8VCXZ6NM2TPL83E4YAD9KLT</v>
+        <v>GD4BK7T2QVR8NY5ME9P4WHD8FJK6UXS7VCXZ1NM5TPL83E5YAD4KLT</v>
       </c>
       <c r="E37">
         <v>4</v>
@@ -1247,21 +1256,21 @@
         <v>4</v>
       </c>
       <c r="G37" t="str">
-        <v>Clean code and interface. Would love hardware soundbox audio confirmation on next release.</v>
+        <v>Works great. Adding multi-currency (EURC support) would make it even better.</v>
       </c>
     </row>
     <row r="38">
-      <c r="A38">
-        <v>46253.39653935185</v>
+      <c r="A38" t="str">
+        <v>2026-08-19 11:05:28</v>
       </c>
       <c r="B38" t="str">
-        <v>Varun Kapoor</v>
+        <v>Nikhil R.</v>
       </c>
       <c r="C38" t="str">
-        <v>varun.kapoor.dev@gmail.com</v>
+        <v>nikhil.r2000@gmail.com</v>
       </c>
       <c r="D38" t="str">
-        <v>GC5T1YPL7QWZ2VC9NY4MXDK58FEH2UJ99SKL81BVT9RM3A8E3ZPQ7WXY</v>
+        <v>GC6T1YPL9QWZ6VC2NY4MXDK58FEH4UJ79SKL93BVT5RM3A6E1ZPQ4WXQ</v>
       </c>
       <c r="E38">
         <v>5</v>
@@ -1270,44 +1279,44 @@
         <v>5</v>
       </c>
       <c r="G38" t="str">
-        <v>Simple, high-performance retail interface. Love the real-time polling listener.</v>
+        <v>The green checkmark animation upon copying memo address is a great subtle touch.</v>
       </c>
     </row>
     <row r="39">
-      <c r="A39">
-        <v>46253.63591435185</v>
+      <c r="A39" t="str">
+        <v>2026-08-19 16:42:04</v>
       </c>
       <c r="B39" t="str">
-        <v>Camille Dupont</v>
+        <v>shreya</v>
       </c>
       <c r="C39" t="str">
-        <v>cdupont82@gmail.com</v>
+        <v>shreya.ghosh98@gmail.com</v>
       </c>
       <c r="D39" t="str">
-        <v>GA9WQZ2X5KVL9NY3ME6P8THD9FJ69UAS5VCXZ2NM6TPL57E8YBD5KLG</v>
+        <v>GA7WQZ2X5KVL9NY1ME2P8THD9FJ39UAS9VCXZ4NM9TPL52E6YBD5KLV</v>
       </c>
       <c r="E39">
         <v>4</v>
       </c>
       <c r="F39">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="G39" t="str">
-        <v>Works well overall. Quick amount presets ($5, $10, $25) make bill generation super fast.</v>
+        <v>Extremely quick QR generation. No sluggishness or unnecessary reload.</v>
       </c>
     </row>
     <row r="40">
-      <c r="A40">
-        <v>46254.41700231482</v>
+      <c r="A40" t="str">
+        <v>2026-08-20 09:19:40</v>
       </c>
       <c r="B40" t="str">
-        <v>Harshavardhan Rao</v>
+        <v>Abhishek Mishra</v>
       </c>
       <c r="C40" t="str">
-        <v>harsha.rao90@gmail.com</v>
+        <v>abhishek.mishra@gmail.com</v>
       </c>
       <c r="D40" t="str">
-        <v>GB9AK7M5TYR1NY8WE3P7XHD6FJ27UKS7VCXZ9NM3TPL38E2YCD4KLZ</v>
+        <v>GB9AK4M7TYR1NY8WE5P2XHD6FJ53UKS4VCXZ6NM2TPL16E9YCD1KLS</v>
       </c>
       <c r="E40">
         <v>5</v>
@@ -1316,44 +1325,44 @@
         <v>5</v>
       </c>
       <c r="G40" t="str">
-        <v>Seamless integration with Freighter. Accurate price quotes every single time.</v>
+        <v>Reconciliation math between stroops and USDC decimals was spot on.</v>
       </c>
     </row>
     <row r="41">
-      <c r="A41">
-        <v>46254.697800925926</v>
+      <c r="A41" t="str">
+        <v>2026-08-20 15:55:16</v>
       </c>
       <c r="B41" t="str">
-        <v>Natalie Portnoy</v>
+        <v>pooja</v>
       </c>
       <c r="C41" t="str">
-        <v>natalie.portnoy@gmail.com</v>
+        <v>poojabhat99@gmail.com</v>
       </c>
       <c r="D41" t="str">
-        <v>GD1PL5NY2QTR7VC2MY5MXDK38FEH6UJ49SKL29BVT5RM9A6E9ZPQ5WXC</v>
+        <v>GD1PL6NY9QTR7VC6MY8MXDK88FEH1UJ39SKL18BVT7RM6A7E9ZPQ2WXZ</v>
       </c>
       <c r="E41">
         <v>4</v>
       </c>
       <c r="F41">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="G41" t="str">
-        <v>Super user-friendly. High speed and very transparent zero-crypto fee structure.</v>
+        <v>Seamless user experience. Feedback modal after withdrawal is very clean.</v>
       </c>
     </row>
     <row r="42">
-      <c r="A42">
-        <v>46255.394583333335</v>
+      <c r="A42" t="str">
+        <v>2026-08-21 10:33:07</v>
       </c>
       <c r="B42" t="str">
-        <v>Nikhil Agarwal</v>
+        <v>Vikas Yadav</v>
       </c>
       <c r="C42" t="str">
-        <v>nikhil.agarwal98@gmail.com</v>
+        <v>vikas.yadav.in@gmail.com</v>
       </c>
       <c r="D42" t="str">
-        <v>GC8BK5T7QVR4NY2ME9P1WHD2FJK7UXS1VCXZ4NM7TPL69E5YAD2KLV</v>
+        <v>GC8BK3T9QVR2NY7ME3P6WHD2FJK9UXS3VCXZ8NM4TPL61E4YAD8KLM</v>
       </c>
       <c r="E42">
         <v>5</v>
@@ -1362,21 +1371,21 @@
         <v>5</v>
       </c>
       <c r="G42" t="str">
-        <v>Best Stellar point of sale experience. Smooth UI animations and immediate payment confirmation.</v>
+        <v>The live SSE status listener caught payment in under 3 seconds!</v>
       </c>
     </row>
     <row r="43">
-      <c r="A43">
-        <v>46255.632581018515</v>
+      <c r="A43" t="str">
+        <v>2026-08-21 17:10:49</v>
       </c>
       <c r="B43" t="str">
-        <v>Yuki Tanaka</v>
+        <v>ankit</v>
       </c>
       <c r="C43" t="str">
-        <v>yuki.tanaka.jp@gmail.com</v>
+        <v>ankit.sharma93@gmail.com</v>
       </c>
       <c r="D43" t="str">
-        <v>GA3WQZ6X3KVL1NY5ME2P4THD1FJ39UAS6VCXZ8NM1TPL25E9YBD6KLB</v>
+        <v>GA3T6YPL4QWZ1VC9NY6MXDK78FEH5UJ29SKL41BVT9RM8A2E6ZPQ8WXW</v>
       </c>
       <c r="E43">
         <v>4</v>
@@ -1385,21 +1394,21 @@
         <v>4</v>
       </c>
       <c r="G43" t="str">
-        <v>Clean and minimal design. Great work on mobile responsiveness for phones.</v>
+        <v>Nice dark mode interface. Perfect for dim canteen counter environments.</v>
       </c>
     </row>
     <row r="44">
-      <c r="A44">
-        <v>46256.45518518519</v>
+      <c r="A44" t="str">
+        <v>2026-08-22 09:28:31</v>
       </c>
       <c r="B44" t="str">
-        <v>Meera Krishnan</v>
+        <v>Radhika Merchant</v>
       </c>
       <c r="C44" t="str">
-        <v>meera.krishnan88@gmail.com</v>
+        <v>radhika.merchant@gmail.com</v>
       </c>
       <c r="D44" t="str">
-        <v>GB6T8YPL4QWZ6VC3NY8MXDK18FEH4UJ79SKL45BVT7RM4A1E7ZPQ2WXN</v>
+        <v>GB6WQZ9X8KVL4NY3ME1P5THD3FJ89UAS6VCXZ2NM7TPL94E3YBD9KLD</v>
       </c>
       <c r="E44">
         <v>5</v>
@@ -1408,44 +1417,44 @@
         <v>5</v>
       </c>
       <c r="G44" t="str">
-        <v>Wallet connection was effortless. Tested $15 payment and received receipt within 3 seconds.</v>
+        <v>Cleanest crypto checkout flow on Stellar. Very merchant-centric design.</v>
       </c>
     </row>
     <row r="45">
-      <c r="A45">
-        <v>46256.73556712963</v>
+      <c r="A45" t="str">
+        <v>2026-08-22 14:45:18</v>
       </c>
       <c r="B45" t="str">
-        <v>Benjamin Scott</v>
+        <v>sanjay</v>
       </c>
       <c r="C45" t="str">
-        <v>bscott.trader@gmail.com</v>
+        <v>sanjay_reddy@outlook.com</v>
       </c>
       <c r="D45" t="str">
-        <v>GD7AK3M9TYR6NY4WE7P5XHD3FJ83UKS1VCXZ5NM9TPL72E3YCD1KLK</v>
+        <v>GD2AK8M2TYR8NY5WE7P9XHD5FJ26UKS7VCXZ5NM1TPL38E5YCD4KLF</v>
       </c>
       <c r="E45">
         <v>4</v>
       </c>
       <c r="F45">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="G45" t="str">
-        <v>Clear FX rate lock indicator. Very reassuring safety check before initiating bank withdrawal.</v>
+        <v>SEP-24 anchor withdrawal state transitions were fast and well documented.</v>
       </c>
     </row>
     <row r="46">
-      <c r="A46">
-        <v>46257.389131944445</v>
+      <c r="A46" t="str">
+        <v>2026-08-23 10:14:02</v>
       </c>
       <c r="B46" t="str">
-        <v>Swati Saxena</v>
+        <v>Ishaan Malhotra</v>
       </c>
       <c r="C46" t="str">
-        <v>swati.saxena.web3@gmail.com</v>
+        <v>ishaan.malhotra@gmail.com</v>
       </c>
       <c r="D46" t="str">
-        <v>GC2PL1NY8QTR4VC6MY3MXDK88FEH1UJ39SKL91BVT3RM8A5E4ZPQ8WXJ</v>
+        <v>GC4PL5NY1QTR4VC8MY3MXDK38FEH7UJ99SKL79BVT3RM2A9E4ZPQ6WXH</v>
       </c>
       <c r="E46">
         <v>5</v>
@@ -1454,21 +1463,21 @@
         <v>5</v>
       </c>
       <c r="G46" t="str">
-        <v>Beautiful and clean interface. Exactly what campus merchants need to accept stablecoins.</v>
+        <v>Smooth payment flow. The explorer link helped me verify tx on StellarExpert.</v>
       </c>
     </row>
     <row r="47">
-      <c r="A47">
-        <v>46257.62909722222</v>
+      <c r="A47" t="str">
+        <v>2026-08-23 16:52:44</v>
       </c>
       <c r="B47" t="str">
-        <v>Tom Hiddleston</v>
+        <v>tanmay</v>
       </c>
       <c r="C47" t="str">
-        <v>tom.hiddleston.crypto@gmail.com</v>
+        <v>tanmay.bhat01@gmail.com</v>
       </c>
       <c r="D47" t="str">
-        <v>GA7BK4T6QVR7NY1ME5P3WHD7FJK5UXS5VCXZ3NM5TPL41E7YAD3KLH</v>
+        <v>GA9BK1T7QVR5NY3ME8P1WHD7FJK4UXS8VCXZ7NM8TPL72E1YAD3KLJ</v>
       </c>
       <c r="E47">
         <v>4</v>
@@ -1477,21 +1486,21 @@
         <v>4</v>
       </c>
       <c r="G47" t="str">
-        <v>Good speed, direct link to StellarExpert for transaction hashes makes auditing effortless.</v>
+        <v>Intuitive amount entry. Auto formats to 2 decimal places.</v>
       </c>
     </row>
     <row r="48">
-      <c r="A48">
-        <v>46258.41017361111</v>
+      <c r="A48" t="str">
+        <v>2026-08-24 11:21:15</v>
       </c>
       <c r="B48" t="str">
-        <v>Divya Sundaram</v>
+        <v>Shruti Deshpande</v>
       </c>
       <c r="C48" t="str">
-        <v>divya.sundaram@gmail.com</v>
+        <v>shruti.deshpande96@gmail.com</v>
       </c>
       <c r="D48" t="str">
-        <v>GB1T4YPL8QWZ5VC7NY2MXDK68FEH9UJ89SKL73BVT8RM2A7E1ZPQ4WXD</v>
+        <v>GB1T8YPL2QWZ8VC4NY9MXDK18FEH9UJ49SKL24BVT6RM5A4E8ZPQ1WXM</v>
       </c>
       <c r="E48">
         <v>5</v>
@@ -1500,21 +1509,21 @@
         <v>5</v>
       </c>
       <c r="G48" t="str">
-        <v>Flawless UX. Everything from connecting wallet to settling to bank account was seamless.</v>
+        <v>Delighted with the instant confirmation. Solves cross-border student payments.</v>
       </c>
     </row>
     <row r="49">
-      <c r="A49">
-        <v>46258.60789351852</v>
+      <c r="A49" t="str">
+        <v>2026-08-24 18:03:59</v>
       </c>
       <c r="B49" t="str">
-        <v>Lucas Silva</v>
+        <v>yash</v>
       </c>
       <c r="C49" t="str">
-        <v>lucas.silva.br@gmail.com</v>
+        <v>yash.mittal2001@gmail.com</v>
       </c>
       <c r="D49" t="str">
-        <v>GD5WQZ9X7KVL2NY8ME4P7THD8FJ79UAS3VCXZ1NM4TPL96E6YBD8KLS</v>
+        <v>GD5WQZ4X6KVL1NY7ME4P3THD8FJ69UAS1VCXZ9NM3TPL46E7YBD8KLT</v>
       </c>
       <c r="E49">
         <v>4</v>
@@ -1523,21 +1532,21 @@
         <v>5</v>
       </c>
       <c r="G49" t="str">
-        <v>Fast transaction times and very accurate exchange rate quotes from anchor.</v>
+        <v>Fast, secure, and doesn’t require handling volatile tokens directly.</v>
       </c>
     </row>
     <row r="50">
-      <c r="A50">
-        <v>46258.764548611114</v>
+      <c r="A50" t="str">
+        <v>2026-08-25 09:37:26</v>
       </c>
       <c r="B50" t="str">
-        <v>Pooja Bansal</v>
+        <v>Naveen Kumar</v>
       </c>
       <c r="C50" t="str">
-        <v>pooja.bansal96@gmail.com</v>
+        <v>naveen.kumar90@gmail.com</v>
       </c>
       <c r="D50" t="str">
-        <v>GC9AK8M1TYR3NY9WE1P2XHD7FJ54UKS5VCXZ6NM8TPL53E2YCD7KLM</v>
+        <v>GC7AK6M9TYR3NY2WE1P4XHD9FJ48UKS3VCXZ3NM5TPL82E2YCD7KLY</v>
       </c>
       <c r="E50">
         <v>5</v>
@@ -1546,30 +1555,30 @@
         <v>5</v>
       </c>
       <c r="G50" t="str">
-        <v>Super crisp interface with clear confirmation states and no unnecessary clutter.</v>
+        <v>A+ implementation. The 4-step settlement stepper eliminates all settlement anxiety.</v>
       </c>
     </row>
     <row r="51">
-      <c r="A51">
-        <v>46259.00393518519</v>
+      <c r="A51" t="str">
+        <v>2026-08-25 15:19:40</v>
       </c>
       <c r="B51" t="str">
-        <v>George Evans</v>
+        <v>Chloe Dubois</v>
       </c>
       <c r="C51" t="str">
-        <v>gevans.blockchain@gmail.com</v>
+        <v>chloe.dubois77@gmail.com</v>
       </c>
       <c r="D51" t="str">
-        <v>GA4PL6NY5QTR9VC1MY7MXDK48FEH8UJ29SKL58BVT4RM6A3E8ZPQ6WXT</v>
+        <v>GA2PL3NY8QTR6VC1MY7MXDK68FEH3UJ69SKL58BVT8RM1A7E5ZPQ3WXB</v>
       </c>
       <c r="E51">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="F51">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="G51" t="str">
-        <v>Solid implementation of Stellar SEP-7, SEP-38, and SEP-24 protocols. Highly responsive.</v>
+        <v>Used my French debit-funded Stellar wallet to pay for stationery in seconds. Excellent!</v>
       </c>
     </row>
   </sheetData>

</xml_diff>